<commit_message>
feat: added orcamento column
</commit_message>
<xml_diff>
--- a/Gestão MEG.xlsx
+++ b/Gestão MEG.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ml0559\Documents\Projetos\node\dash_melhorias\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ml0559\Documents\Projetos\node\dash_melhorias\dash_melhorias\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FACCDF36-7569-4A3D-AC66-1D950646E575}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B74A8211-5F11-41B5-A3FB-D88101F47C25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4499" uniqueCount="530">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4500" uniqueCount="531">
   <si>
     <t>ID do plano</t>
   </si>
@@ -1634,6 +1634,9 @@
   </si>
   <si>
     <t>Tarefas Antigas</t>
+  </si>
+  <si>
+    <t>Orçamento</t>
   </si>
 </sst>
 </file>
@@ -2070,7 +2073,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:S124"/>
+  <dimension ref="A1:T125"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.875" customWidth="1"/>
@@ -2089,9 +2092,10 @@
     <col min="15" max="15" width="32.875" customWidth="1"/>
     <col min="16" max="16" width="41.625" customWidth="1"/>
     <col min="17" max="19" width="32.875" customWidth="1"/>
+    <col min="20" max="20" width="13.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -2149,8 +2153,11 @@
       <c r="S1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T1" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>25</v>
       </c>
@@ -2206,8 +2213,11 @@
       <c r="R2" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T2">
+        <v>880.64</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>38</v>
       </c>
@@ -2263,8 +2273,11 @@
       <c r="R3" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T3">
+        <v>321.55</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>44</v>
       </c>
@@ -2320,8 +2333,11 @@
       <c r="R4" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T4">
+        <v>560.77</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>49</v>
       </c>
@@ -2377,8 +2393,11 @@
       <c r="R5" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T5">
+        <v>755.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>51</v>
       </c>
@@ -2434,8 +2453,11 @@
       <c r="R6" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T6">
+        <v>349.29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>53</v>
       </c>
@@ -2491,8 +2513,11 @@
       <c r="R7" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T7">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>55</v>
       </c>
@@ -2548,8 +2573,11 @@
       <c r="R8" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T8">
+        <v>502.98</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>57</v>
       </c>
@@ -2605,8 +2633,11 @@
       <c r="R9" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T9">
+        <v>110.46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>59</v>
       </c>
@@ -2662,8 +2693,11 @@
       <c r="R10" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T10">
+        <v>32.19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>62</v>
       </c>
@@ -2719,8 +2753,11 @@
       <c r="R11" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T11">
+        <v>391.93</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>70</v>
       </c>
@@ -2776,8 +2813,11 @@
       <c r="R12" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T12">
+        <v>52.13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>74</v>
       </c>
@@ -2833,8 +2873,11 @@
       <c r="R13" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T13">
+        <v>173.06</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>77</v>
       </c>
@@ -2890,8 +2933,11 @@
       <c r="R14" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T14">
+        <v>96.29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>83</v>
       </c>
@@ -2950,8 +2996,11 @@
       <c r="S15" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T15">
+        <v>318.55</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>86</v>
       </c>
@@ -3007,8 +3056,11 @@
       <c r="R16" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T16">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>90</v>
       </c>
@@ -3064,8 +3116,11 @@
       <c r="R17" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T17">
+        <v>274.44</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>96</v>
       </c>
@@ -3121,8 +3176,11 @@
       <c r="R18" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T18">
+        <v>210.98</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>100</v>
       </c>
@@ -3178,8 +3236,11 @@
       <c r="R19" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T19">
+        <v>389.75</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>102</v>
       </c>
@@ -3235,8 +3296,11 @@
       <c r="R20" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T20">
+        <v>499.61</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>105</v>
       </c>
@@ -3292,8 +3356,11 @@
       <c r="R21" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T21">
+        <v>612.74</v>
+      </c>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>108</v>
       </c>
@@ -3349,8 +3416,11 @@
       <c r="R22" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T22">
+        <v>273.08</v>
+      </c>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>114</v>
       </c>
@@ -3406,8 +3476,11 @@
       <c r="R23" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T23">
+        <v>793.53</v>
+      </c>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>116</v>
       </c>
@@ -3463,8 +3536,11 @@
       <c r="R24" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T24">
+        <v>987.87</v>
+      </c>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>119</v>
       </c>
@@ -3520,8 +3596,11 @@
       <c r="R25" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T25">
+        <v>74.97</v>
+      </c>
+    </row>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>132</v>
       </c>
@@ -3577,8 +3656,11 @@
       <c r="R26" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T26">
+        <v>426.94</v>
+      </c>
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>141</v>
       </c>
@@ -3634,8 +3716,11 @@
       <c r="R27" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T27">
+        <v>244.88</v>
+      </c>
+    </row>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>148</v>
       </c>
@@ -3691,8 +3776,11 @@
       <c r="R28" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T28">
+        <v>273.43</v>
+      </c>
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>153</v>
       </c>
@@ -3748,8 +3836,11 @@
       <c r="R29" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T29">
+        <v>719.5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>157</v>
       </c>
@@ -3805,8 +3896,11 @@
       <c r="R30" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T30">
+        <v>732.63</v>
+      </c>
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>162</v>
       </c>
@@ -3865,8 +3959,11 @@
       <c r="S31" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T31">
+        <v>451.23</v>
+      </c>
+    </row>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>169</v>
       </c>
@@ -3925,8 +4022,11 @@
       <c r="S32" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T32">
+        <v>475.39</v>
+      </c>
+    </row>
+    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>175</v>
       </c>
@@ -3982,8 +4082,11 @@
       <c r="R33" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T33">
+        <v>396.3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>180</v>
       </c>
@@ -4039,8 +4142,11 @@
       <c r="R34" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T34">
+        <v>102.4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>182</v>
       </c>
@@ -4096,8 +4202,11 @@
       <c r="R35" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T35">
+        <v>960.52</v>
+      </c>
+    </row>
+    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>184</v>
       </c>
@@ -4153,8 +4262,11 @@
       <c r="R36" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T36">
+        <v>503.93</v>
+      </c>
+    </row>
+    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>190</v>
       </c>
@@ -4210,8 +4322,11 @@
       <c r="R37" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T37">
+        <v>618.85</v>
+      </c>
+    </row>
+    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>195</v>
       </c>
@@ -4267,8 +4382,11 @@
       <c r="R38" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T38">
+        <v>194.13</v>
+      </c>
+    </row>
+    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>197</v>
       </c>
@@ -4324,8 +4442,11 @@
       <c r="R39" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T39">
+        <v>505.12</v>
+      </c>
+    </row>
+    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>205</v>
       </c>
@@ -4381,8 +4502,11 @@
       <c r="R40" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T40">
+        <v>107.76</v>
+      </c>
+    </row>
+    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>210</v>
       </c>
@@ -4441,8 +4565,11 @@
       <c r="S41" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T41">
+        <v>87.21</v>
+      </c>
+    </row>
+    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>214</v>
       </c>
@@ -4498,8 +4625,11 @@
       <c r="R42" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T42">
+        <v>511.17</v>
+      </c>
+    </row>
+    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>219</v>
       </c>
@@ -4555,8 +4685,11 @@
       <c r="R43" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T43">
+        <v>939.14</v>
+      </c>
+    </row>
+    <row r="44" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>221</v>
       </c>
@@ -4612,8 +4745,11 @@
       <c r="R44" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T44">
+        <v>204.8</v>
+      </c>
+    </row>
+    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>222</v>
       </c>
@@ -4669,8 +4805,11 @@
       <c r="R45" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T45">
+        <v>805.18</v>
+      </c>
+    </row>
+    <row r="46" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>224</v>
       </c>
@@ -4726,8 +4865,11 @@
       <c r="R46" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T46">
+        <v>100.58</v>
+      </c>
+    </row>
+    <row r="47" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>226</v>
       </c>
@@ -4783,8 +4925,11 @@
       <c r="R47" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T47">
+        <v>588.29999999999995</v>
+      </c>
+    </row>
+    <row r="48" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>228</v>
       </c>
@@ -4840,8 +4985,11 @@
       <c r="R48" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T48">
+        <v>535.16</v>
+      </c>
+    </row>
+    <row r="49" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>233</v>
       </c>
@@ -4897,8 +5045,11 @@
       <c r="R49" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T49">
+        <v>432.77</v>
+      </c>
+    </row>
+    <row r="50" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>238</v>
       </c>
@@ -4954,8 +5105,11 @@
       <c r="R50" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T50">
+        <v>463.31</v>
+      </c>
+    </row>
+    <row r="51" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>240</v>
       </c>
@@ -5011,8 +5165,11 @@
       <c r="R51" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T51">
+        <v>438.74</v>
+      </c>
+    </row>
+    <row r="52" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>242</v>
       </c>
@@ -5068,8 +5225,11 @@
       <c r="R52" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T52">
+        <v>815.71</v>
+      </c>
+    </row>
+    <row r="53" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>245</v>
       </c>
@@ -5125,8 +5285,11 @@
       <c r="R53" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T53">
+        <v>312.45</v>
+      </c>
+    </row>
+    <row r="54" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>247</v>
       </c>
@@ -5182,8 +5345,11 @@
       <c r="R54" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T54">
+        <v>45.21</v>
+      </c>
+    </row>
+    <row r="55" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>250</v>
       </c>
@@ -5239,8 +5405,11 @@
       <c r="R55" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T55">
+        <v>50.34</v>
+      </c>
+    </row>
+    <row r="56" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>253</v>
       </c>
@@ -5296,8 +5465,11 @@
       <c r="R56" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T56">
+        <v>536.25</v>
+      </c>
+    </row>
+    <row r="57" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>256</v>
       </c>
@@ -5353,8 +5525,11 @@
       <c r="R57" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="58" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T57">
+        <v>904.74</v>
+      </c>
+    </row>
+    <row r="58" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>258</v>
       </c>
@@ -5413,8 +5588,11 @@
       <c r="S58" t="s">
         <v>261</v>
       </c>
-    </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T58">
+        <v>695.57</v>
+      </c>
+    </row>
+    <row r="59" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>262</v>
       </c>
@@ -5470,8 +5648,11 @@
       <c r="R59" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T59">
+        <v>379.62</v>
+      </c>
+    </row>
+    <row r="60" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>266</v>
       </c>
@@ -5530,8 +5711,11 @@
       <c r="S60" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="61" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T60">
+        <v>290.77</v>
+      </c>
+    </row>
+    <row r="61" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>271</v>
       </c>
@@ -5587,8 +5771,11 @@
       <c r="R61" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="62" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T61">
+        <v>917.2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>273</v>
       </c>
@@ -5644,8 +5831,11 @@
       <c r="R62" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T62">
+        <v>465.7</v>
+      </c>
+    </row>
+    <row r="63" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>275</v>
       </c>
@@ -5701,8 +5891,11 @@
       <c r="R63" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T63">
+        <v>936.21</v>
+      </c>
+    </row>
+    <row r="64" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>278</v>
       </c>
@@ -5758,8 +5951,11 @@
       <c r="R64" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="65" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T64">
+        <v>456.62</v>
+      </c>
+    </row>
+    <row r="65" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>280</v>
       </c>
@@ -5815,8 +6011,11 @@
       <c r="R65" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="66" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T65">
+        <v>879.46</v>
+      </c>
+    </row>
+    <row r="66" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>283</v>
       </c>
@@ -5872,8 +6071,11 @@
       <c r="R66" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="67" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T66">
+        <v>75.989999999999995</v>
+      </c>
+    </row>
+    <row r="67" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>287</v>
       </c>
@@ -5929,8 +6131,11 @@
       <c r="R67" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="68" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T67">
+        <v>646.13</v>
+      </c>
+    </row>
+    <row r="68" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>290</v>
       </c>
@@ -5986,8 +6191,11 @@
       <c r="R68" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="69" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T68">
+        <v>23.01</v>
+      </c>
+    </row>
+    <row r="69" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>294</v>
       </c>
@@ -6043,8 +6251,11 @@
       <c r="R69" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="70" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T69">
+        <v>315.31</v>
+      </c>
+    </row>
+    <row r="70" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>296</v>
       </c>
@@ -6100,8 +6311,11 @@
       <c r="R70" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="71" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T70">
+        <v>947.2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>300</v>
       </c>
@@ -6157,8 +6371,11 @@
       <c r="R71" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="72" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T71">
+        <v>522.23</v>
+      </c>
+    </row>
+    <row r="72" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>305</v>
       </c>
@@ -6214,8 +6431,11 @@
       <c r="R72" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="73" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T72">
+        <v>627.75</v>
+      </c>
+    </row>
+    <row r="73" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>309</v>
       </c>
@@ -6271,8 +6491,11 @@
       <c r="R73" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="74" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T73">
+        <v>8.67</v>
+      </c>
+    </row>
+    <row r="74" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>311</v>
       </c>
@@ -6328,8 +6551,11 @@
       <c r="R74" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="75" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T74">
+        <v>502.3</v>
+      </c>
+    </row>
+    <row r="75" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>314</v>
       </c>
@@ -6385,8 +6611,11 @@
       <c r="R75" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="76" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T75">
+        <v>127.34</v>
+      </c>
+    </row>
+    <row r="76" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>316</v>
       </c>
@@ -6442,8 +6671,11 @@
       <c r="R76" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="77" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T76">
+        <v>280.72000000000003</v>
+      </c>
+    </row>
+    <row r="77" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>320</v>
       </c>
@@ -6499,8 +6731,11 @@
       <c r="R77" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="78" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T77">
+        <v>52.23</v>
+      </c>
+    </row>
+    <row r="78" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>323</v>
       </c>
@@ -6559,8 +6794,11 @@
       <c r="S78" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="79" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T78">
+        <v>976.11</v>
+      </c>
+    </row>
+    <row r="79" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>326</v>
       </c>
@@ -6616,8 +6854,11 @@
       <c r="R79" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="80" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T79">
+        <v>426.08</v>
+      </c>
+    </row>
+    <row r="80" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>329</v>
       </c>
@@ -6673,8 +6914,11 @@
       <c r="R80" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="81" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T80">
+        <v>499.33</v>
+      </c>
+    </row>
+    <row r="81" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>332</v>
       </c>
@@ -6730,8 +6974,11 @@
       <c r="R81" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="82" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T81">
+        <v>705.43</v>
+      </c>
+    </row>
+    <row r="82" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>339</v>
       </c>
@@ -6787,8 +7034,11 @@
       <c r="R82" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="83" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T82">
+        <v>204.85</v>
+      </c>
+    </row>
+    <row r="83" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>341</v>
       </c>
@@ -6844,8 +7094,11 @@
       <c r="R83" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="84" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T83">
+        <v>592.49</v>
+      </c>
+    </row>
+    <row r="84" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>343</v>
       </c>
@@ -6901,8 +7154,11 @@
       <c r="R84" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="85" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T84">
+        <v>645.91999999999996</v>
+      </c>
+    </row>
+    <row r="85" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>345</v>
       </c>
@@ -6958,8 +7214,11 @@
       <c r="R85" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="86" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T85">
+        <v>301.13</v>
+      </c>
+    </row>
+    <row r="86" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>347</v>
       </c>
@@ -7015,8 +7274,11 @@
       <c r="R86" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="87" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T86">
+        <v>43.83</v>
+      </c>
+    </row>
+    <row r="87" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>349</v>
       </c>
@@ -7072,8 +7334,11 @@
       <c r="R87" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="88" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T87">
+        <v>26.47</v>
+      </c>
+    </row>
+    <row r="88" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>351</v>
       </c>
@@ -7129,8 +7394,11 @@
       <c r="R88" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="89" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T88">
+        <v>776.96</v>
+      </c>
+    </row>
+    <row r="89" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>353</v>
       </c>
@@ -7186,8 +7454,11 @@
       <c r="R89" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="90" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T89">
+        <v>305.23</v>
+      </c>
+    </row>
+    <row r="90" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>355</v>
       </c>
@@ -7243,8 +7514,11 @@
       <c r="R90" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="91" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T90">
+        <v>456.21</v>
+      </c>
+    </row>
+    <row r="91" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>357</v>
       </c>
@@ -7300,8 +7574,11 @@
       <c r="R91" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="92" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T91">
+        <v>715.98</v>
+      </c>
+    </row>
+    <row r="92" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>361</v>
       </c>
@@ -7357,8 +7634,11 @@
       <c r="R92" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="93" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T92">
+        <v>671.96</v>
+      </c>
+    </row>
+    <row r="93" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>363</v>
       </c>
@@ -7414,8 +7694,11 @@
       <c r="R93" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="94" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T93">
+        <v>516.5</v>
+      </c>
+    </row>
+    <row r="94" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>365</v>
       </c>
@@ -7471,8 +7754,11 @@
       <c r="R94" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="95" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T94">
+        <v>34.49</v>
+      </c>
+    </row>
+    <row r="95" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>369</v>
       </c>
@@ -7528,8 +7814,11 @@
       <c r="R95" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="96" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T95">
+        <v>504.98</v>
+      </c>
+    </row>
+    <row r="96" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>371</v>
       </c>
@@ -7585,8 +7874,11 @@
       <c r="R96" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="97" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T96">
+        <v>990.77</v>
+      </c>
+    </row>
+    <row r="97" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>373</v>
       </c>
@@ -7642,8 +7934,11 @@
       <c r="R97" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="98" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T97">
+        <v>9.8000000000000007</v>
+      </c>
+    </row>
+    <row r="98" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>375</v>
       </c>
@@ -7699,8 +7994,11 @@
       <c r="R98" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="99" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T98">
+        <v>833.24</v>
+      </c>
+    </row>
+    <row r="99" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>379</v>
       </c>
@@ -7756,8 +8054,11 @@
       <c r="R99" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="100" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T99">
+        <v>784.14</v>
+      </c>
+    </row>
+    <row r="100" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>383</v>
       </c>
@@ -7813,8 +8114,11 @@
       <c r="R100" t="s">
         <v>387</v>
       </c>
-    </row>
-    <row r="101" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T100">
+        <v>764.24</v>
+      </c>
+    </row>
+    <row r="101" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>388</v>
       </c>
@@ -7870,8 +8174,11 @@
       <c r="R101" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="102" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T101">
+        <v>16.66</v>
+      </c>
+    </row>
+    <row r="102" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>391</v>
       </c>
@@ -7927,8 +8234,11 @@
       <c r="R102" t="s">
         <v>387</v>
       </c>
-    </row>
-    <row r="103" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T102">
+        <v>556.80999999999995</v>
+      </c>
+    </row>
+    <row r="103" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>395</v>
       </c>
@@ -7984,8 +8294,11 @@
       <c r="R103" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="104" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T103">
+        <v>436.44</v>
+      </c>
+    </row>
+    <row r="104" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>397</v>
       </c>
@@ -8041,8 +8354,11 @@
       <c r="R104" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="105" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T104">
+        <v>433.95</v>
+      </c>
+    </row>
+    <row r="105" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>399</v>
       </c>
@@ -8098,8 +8414,11 @@
       <c r="R105" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="106" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T105">
+        <v>428.58</v>
+      </c>
+    </row>
+    <row r="106" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>405</v>
       </c>
@@ -8155,8 +8474,11 @@
       <c r="R106" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="107" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T106">
+        <v>511.6</v>
+      </c>
+    </row>
+    <row r="107" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>407</v>
       </c>
@@ -8212,8 +8534,11 @@
       <c r="R107" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="108" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T107">
+        <v>994.97</v>
+      </c>
+    </row>
+    <row r="108" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>411</v>
       </c>
@@ -8269,8 +8594,11 @@
       <c r="R108" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="109" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T108">
+        <v>662.67</v>
+      </c>
+    </row>
+    <row r="109" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>413</v>
       </c>
@@ -8326,8 +8654,11 @@
       <c r="R109" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="110" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T109">
+        <v>168.18</v>
+      </c>
+    </row>
+    <row r="110" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>415</v>
       </c>
@@ -8383,8 +8714,11 @@
       <c r="R110" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="111" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T110">
+        <v>631.94000000000005</v>
+      </c>
+    </row>
+    <row r="111" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>417</v>
       </c>
@@ -8440,8 +8774,11 @@
       <c r="R111" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="112" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T111">
+        <v>439.02</v>
+      </c>
+    </row>
+    <row r="112" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>420</v>
       </c>
@@ -8497,8 +8834,11 @@
       <c r="R112" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="113" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T112">
+        <v>187.59</v>
+      </c>
+    </row>
+    <row r="113" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>423</v>
       </c>
@@ -8554,8 +8894,11 @@
       <c r="R113" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="114" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T113">
+        <v>550.34</v>
+      </c>
+    </row>
+    <row r="114" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>427</v>
       </c>
@@ -8611,8 +8954,11 @@
       <c r="R114" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="115" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T114">
+        <v>339.28</v>
+      </c>
+    </row>
+    <row r="115" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>429</v>
       </c>
@@ -8668,8 +9014,11 @@
       <c r="R115" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="116" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T115">
+        <v>316.27999999999997</v>
+      </c>
+    </row>
+    <row r="116" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>432</v>
       </c>
@@ -8725,8 +9074,11 @@
       <c r="R116" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="117" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T116">
+        <v>859.87</v>
+      </c>
+    </row>
+    <row r="117" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>434</v>
       </c>
@@ -8782,8 +9134,11 @@
       <c r="R117" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="118" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T117">
+        <v>442.41</v>
+      </c>
+    </row>
+    <row r="118" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>436</v>
       </c>
@@ -8839,8 +9194,11 @@
       <c r="R118" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="119" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T118">
+        <v>67.64</v>
+      </c>
+    </row>
+    <row r="119" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>438</v>
       </c>
@@ -8896,8 +9254,11 @@
       <c r="R119" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="120" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T119">
+        <v>244.2</v>
+      </c>
+    </row>
+    <row r="120" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>442</v>
       </c>
@@ -8953,8 +9314,11 @@
       <c r="R120" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="121" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T120">
+        <v>64.97</v>
+      </c>
+    </row>
+    <row r="121" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>446</v>
       </c>
@@ -9010,8 +9374,11 @@
       <c r="R121" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="122" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T121">
+        <v>671.95</v>
+      </c>
+    </row>
+    <row r="122" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>449</v>
       </c>
@@ -9067,8 +9434,11 @@
       <c r="R122" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="123" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T122">
+        <v>115.53</v>
+      </c>
+    </row>
+    <row r="123" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>452</v>
       </c>
@@ -9124,8 +9494,11 @@
       <c r="R123" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="124" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="T123">
+        <v>730.66</v>
+      </c>
+    </row>
+    <row r="124" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>454</v>
       </c>
@@ -9180,6 +9553,14 @@
       </c>
       <c r="R124" t="s">
         <v>28</v>
+      </c>
+      <c r="T124">
+        <v>7.44</v>
+      </c>
+    </row>
+    <row r="125" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="T125">
+        <v>565.41999999999996</v>
       </c>
     </row>
   </sheetData>

</xml_diff>